<commit_message>
Use 7w / 7-11m age labels in comments and README
- Replace "peripubertal" / "young adult" with 7w (7-week-old) and
  7-11m (7-11-month-old) in script comments, the Script 10 README and
  the main README; group codes (e.g. ABF, YBF) and code are unchanged
- Script 1 header: explain the A/Y group codes
- Script 8: rename contrast script to Script8_age_sex_and_age_region_interaction.R
- Script 5: region GSEA workbook sheet order (peri > top before peri < top)
</commit_message>
<xml_diff>
--- a/Script_5_single_factor_pathway/region_vs_region_GSEA/Supplementary_table_region_vs_region_single_factor_GSEA.xlsx
+++ b/Script_5_single_factor_pathway/region_vs_region_GSEA/Supplementary_table_region_vs_region_single_factor_GSEA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/outobi/Downloads/final analysis/final code/Script_5_single_factor_pathway/region_vs_region_GSEA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1F7C4F-8064-574E-82E5-187C3C78F35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D69D838-17EB-894F-8D47-7D44EFD98D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="39120" yWindow="2120" windowWidth="27240" windowHeight="16440" firstSheet="1" activeTab="8" xr2:uid="{D5BAC588-A04A-2545-A7AC-5EE0BDE63D5D}"/>
+    <workbookView xWindow="5320" yWindow="2360" windowWidth="27240" windowHeight="16440" firstSheet="1" activeTab="6" xr2:uid="{D5BAC588-A04A-2545-A7AC-5EE0BDE63D5D}"/>
   </bookViews>
   <sheets>
     <sheet name="GO bottom &lt; central" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,8 @@
     <sheet name="GO central &gt; top" sheetId="6" r:id="rId4"/>
     <sheet name="Reactome central &gt; top" sheetId="7" r:id="rId5"/>
     <sheet name="Reactome central &lt; top" sheetId="10" r:id="rId6"/>
-    <sheet name="GO peri &lt; top" sheetId="8" r:id="rId7"/>
-    <sheet name="GO peri &gt; top" sheetId="11" r:id="rId8"/>
+    <sheet name="GO peri &gt; top" sheetId="11" r:id="rId7"/>
+    <sheet name="GO peri &lt; top" sheetId="8" r:id="rId8"/>
     <sheet name="Reactome peri &lt; top" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -3238,6 +3238,81 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F2296F-3135-8A48-9161-4D0CDCD7B5C9}">
+  <dimension ref="A1:J2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
+        <v>108</v>
+      </c>
+      <c r="C2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D2">
+        <v>17</v>
+      </c>
+      <c r="E2">
+        <v>13</v>
+      </c>
+      <c r="F2">
+        <v>0.73416999999999999</v>
+      </c>
+      <c r="G2">
+        <v>1.8957999999999999</v>
+      </c>
+      <c r="H2">
+        <v>1.6949000000000001E-3</v>
+      </c>
+      <c r="I2">
+        <v>2.2218000000000002E-2</v>
+      </c>
+      <c r="J2">
+        <f t="shared" ref="J2" si="0">-LOG10(I2)</f>
+        <v>1.6532950375669138</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{523E033A-0F74-8942-A7A4-93E45C5623B4}">
   <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -3705,81 +3780,6 @@
       <c r="J14">
         <f t="shared" si="0"/>
         <v>15.657577319177793</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F2296F-3135-8A48-9161-4D0CDCD7B5C9}">
-  <dimension ref="A1:J2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D2">
-        <v>17</v>
-      </c>
-      <c r="E2">
-        <v>13</v>
-      </c>
-      <c r="F2">
-        <v>0.73416999999999999</v>
-      </c>
-      <c r="G2">
-        <v>1.8957999999999999</v>
-      </c>
-      <c r="H2">
-        <v>1.6949000000000001E-3</v>
-      </c>
-      <c r="I2">
-        <v>2.2218000000000002E-2</v>
-      </c>
-      <c r="J2">
-        <f t="shared" ref="J2" si="0">-LOG10(I2)</f>
-        <v>1.6532950375669138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>